<commit_message>
fix: replace Dune Sound relationship
</commit_message>
<xml_diff>
--- a/outputs/01a007e0-b631-7ca1-a18c-9f6e6ff6ff29/VM-563-Sound-Play-Final-Review.xlsx
+++ b/outputs/01a007e0-b631-7ca1-a18c-9f6e6ff6ff29/VM-563-Sound-Play-Final-Review.xlsx
@@ -2,43 +2,43 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 W White" sheetId="1" r:id="R1d6aa310976343d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 U Blue" sheetId="2" r:id="R0a858f890fea4c68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 B Black" sheetId="3" r:id="Reb4422a7d6544e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 R Red" sheetId="4" r:id="R70d4e58e2c894ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 G Green" sheetId="5" r:id="R93c0fab4d2b2409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 WU Azorius Senate" sheetId="6" r:id="R07f01257bc78457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 UB House Dimir" sheetId="7" r:id="R36cf815cf9eb460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 BR Cult of Rakdos" sheetId="8" r:id="Rc5720e52f0374a91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 RG Gruul Clans" sheetId="9" r:id="Rd9a715e357044433"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 WG Selesnya Conclave" sheetId="10" r:id="Rc3590545ae8b4a47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 WB Orzhov Syndicate" sheetId="11" r:id="R33dcef19d0f549d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 UR Izzet League" sheetId="12" r:id="Ref37a89beac44bd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 BG Golgari Swarm" sheetId="13" r:id="Rb0898754bcb9497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 WR Boros Legion" sheetId="14" r:id="R27a7775168a44576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 UG Simic Combine" sheetId="15" r:id="R69c7cc2564504b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 SILVERQUILL Silverquill Coll" sheetId="16" r:id="Re7adbf0e9510406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 PRISMARI Prismari College" sheetId="17" r:id="Rfff55762e66d41a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 WITHERBLOOM Witherbloom Coll" sheetId="18" r:id="Reb7ed26098674d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 LOREHOLD Lorehold College" sheetId="19" r:id="R83cd9edd75144ccb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 QUANDRIX Quandrix College" sheetId="20" r:id="R760b013fffb64fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 BANT Bant" sheetId="21" r:id="R1f84445450614b54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 ESPER Esper" sheetId="22" r:id="Rbf4bbb26e5d9400d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 GRIXIS Grixis" sheetId="23" r:id="R273fb7fbd07a4d05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 JUND Jund" sheetId="24" r:id="Rf1bba22dffe44e68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 NAYA Naya" sheetId="25" r:id="R35d7788f194d4409"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26 ABZAN Abzan Houses" sheetId="26" r:id="Rf4ce86c3112b4cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27 JESKAI Jeskai Way" sheetId="27" r:id="R7d652fedf6664891"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28 SULTAI Sultai Brood" sheetId="28" r:id="R318ec271064c4b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29 MARDU Mardu Horde" sheetId="29" r:id="R548c0c8da80e421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30 TEMUR Temur Frontier" sheetId="30" r:id="Rb338ac1cdc654e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31 YORE Yore - Artifice" sheetId="31" r:id="Redb0e6b90540469f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32 GLINT Glint - Chaos" sheetId="32" r:id="Rd34ee49ba00c4c10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="33 DUNE Dune - Aggression" sheetId="33" r:id="R691d6e10179648bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34 INK Ink - Altruism" sheetId="34" r:id="R741784717013426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="35 WITCH Witch - Growth" sheetId="35" r:id="R07c4f20504d140e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36 WUBRG Five-Color - WUBRG" sheetId="36" r:id="Rfabffeb9a4c84ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="37 COLORLESS Colorless" sheetId="37" r:id="Rdfbd7a072ce04e92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 W White" sheetId="1" r:id="R2d854ff097a14939"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 U Blue" sheetId="2" r:id="R5d68f6693bf14b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 B Black" sheetId="3" r:id="Rdf99822e4abf455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 R Red" sheetId="4" r:id="R24a7915c590f41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 G Green" sheetId="5" r:id="Ra3ab4ff7c4d544b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 WU Azorius Senate" sheetId="6" r:id="Rbbf47847f7084232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 UB House Dimir" sheetId="7" r:id="R52ca826a7a4b4c6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 BR Cult of Rakdos" sheetId="8" r:id="Redc436529ab34f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 RG Gruul Clans" sheetId="9" r:id="R089c8ce1abbd4b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 WG Selesnya Conclave" sheetId="10" r:id="R412b01fafeb34f27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 WB Orzhov Syndicate" sheetId="11" r:id="R7498057c547d488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 UR Izzet League" sheetId="12" r:id="Re0cbbe95d6dc43ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 BG Golgari Swarm" sheetId="13" r:id="R203434442a304679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 WR Boros Legion" sheetId="14" r:id="R789b2c15b993400e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 UG Simic Combine" sheetId="15" r:id="R75ed416ad5b44ea4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 SILVERQUILL Silverquill Coll" sheetId="16" r:id="Rd04682041df14526"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 PRISMARI Prismari College" sheetId="17" r:id="R87d4043aaf414cc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 WITHERBLOOM Witherbloom Coll" sheetId="18" r:id="R309aef839c014a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 LOREHOLD Lorehold College" sheetId="19" r:id="R53a354ffe5644432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 QUANDRIX Quandrix College" sheetId="20" r:id="Rc26fd43e1dcd4d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 BANT Bant" sheetId="21" r:id="R5d51155d7a4d42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 ESPER Esper" sheetId="22" r:id="Rc3cc79bb75d442aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 GRIXIS Grixis" sheetId="23" r:id="Rb09f2ba593a44515"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 JUND Jund" sheetId="24" r:id="R65e9a09d8ece42a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 NAYA Naya" sheetId="25" r:id="Ra16763650ac745df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26 ABZAN Abzan Houses" sheetId="26" r:id="R5e95dbb77f59406a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27 JESKAI Jeskai Way" sheetId="27" r:id="R1cf0203007914b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28 SULTAI Sultai Brood" sheetId="28" r:id="R2e840dbaf1ff4069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29 MARDU Mardu Horde" sheetId="29" r:id="R1f608c35172346ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30 TEMUR Temur Frontier" sheetId="30" r:id="R653447a713fc4449"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31 YORE Yore - Artifice" sheetId="31" r:id="R304e34a20f184d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32 GLINT Glint - Chaos" sheetId="32" r:id="R0bbd00810d73455f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="33 DUNE Dune - Aggression" sheetId="33" r:id="R92878e69dba94e11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34 INK Ink - Altruism" sheetId="34" r:id="R95d5373a531e4c8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="35 WITCH Witch - Growth" sheetId="35" r:id="Rd409e8b2b9834b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36 WUBRG Five-Color - WUBRG" sheetId="36" r:id="R12d4d8b5a02d4fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="37 COLORLESS Colorless" sheetId="37" r:id="R9327683fc8b948b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -234,7 +234,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -245,7 +245,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -256,7 +256,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -267,7 +267,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -278,7 +278,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -289,7 +289,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -300,7 +300,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -311,7 +311,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -322,7 +322,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -333,7 +333,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -344,7 +344,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -355,7 +355,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -366,7 +366,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -377,7 +377,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -388,7 +388,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +399,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +410,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -421,7 +421,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -432,7 +432,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -443,7 +443,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -454,7 +454,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -465,7 +465,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -476,7 +476,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -487,7 +487,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -498,7 +498,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -509,7 +509,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -520,7 +520,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -531,7 +531,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -542,7 +542,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -553,7 +553,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -564,7 +564,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -575,7 +575,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -586,7 +586,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -597,7 +597,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -608,7 +608,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -619,7 +619,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -630,7 +630,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -1721,7 +1721,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd06cd346c48c4fa3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd0001d15d845408f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1917,7 +1917,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ddc743d521942d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80469c784b8c4cf9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2170,7 +2170,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52b8079e58184b04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R744a65c07ddd427d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2395,7 +2395,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3b2ce96d2e4aed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c398ed79cac429c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2588,7 +2588,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61494add12344e54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea42d1b37d4743b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2841,7 +2841,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R861e9040b5b0461e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2513980a243b4c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3036,7 +3036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2edd57d54484427a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80774a489f234545"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3230,7 +3230,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R285d023ec05a4124"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R592762f522e740d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3423,7 +3423,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfa42e40e20149e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51a16d0e157b4150"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3617,7 +3617,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9abf1ba154f4c25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46afe1b09f8c4bae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3842,7 +3842,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cde141893ae4b8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8605e5a5839747d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4036,7 +4036,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f7639c4aded48d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02becbb9c0ea457e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4230,7 +4230,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R145681225d3446a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7da470422ee74ebc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4423,7 +4423,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd06de1023aaa4148"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb49e8c2eb2b44359"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4616,7 +4616,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda5f34ac16924add"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad6eabc6008d4a26"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4811,7 +4811,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R80ee3e2baeff4906"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d266db7d8ad49f6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5004,7 +5004,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ed7da47015457a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9309958f28dd4b36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5197,7 +5197,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f26122205684ef7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Redc26b065c424271"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5392,7 +5392,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40ab6f15afe64790"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R831136021b7645a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5585,7 +5585,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79e6be8c8bed42e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2482a81088a44fea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5779,7 +5779,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reafe6d6c88da4baa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d73cc38fdba4b27"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5974,7 +5974,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f81615157dc494d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dedcfcb5ec04c08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6167,7 +6167,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc467c2b15ab24a51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R026845868d0e4c06"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6361,7 +6361,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R072d8880f4dc4e37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaa16722822b48b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6556,7 +6556,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad62349f6a3d4743"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4e55850e81f4590"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6751,7 +6751,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba81e647858447c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c082c1ba0304206"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6876,32 +6876,34 @@
     </x:row>
     <x:row r="6" ht="94.5" customHeight="1">
       <x:c r="A6" s="21" t="str">
-        <x:v>Scour from Existence</x:v>
+        <x:v>Dune-Brood Nephilim</x:v>
       </x:c>
       <x:c r="B6" s="21" t="str">
         <x:v>Cards That Sound Like This</x:v>
       </x:c>
       <x:c r="C6" s="20" t="str">
+        <x:v>When it awoke, it spawned nameless thousands to herald its arrival.</x:v>
+      </x:c>
+      <x:c r="D6" s="20" t="str">
+        <x:v>The “nameless thousands” become literal when Dune-Brood connects: every land you control adds another Sand token. That multiplying surge gives Dune's physical momentum a different voice from Aurelia's front-line command.</x:v>
+      </x:c>
+      <x:c r="E6" s="20" t="str">
         <x:v>"Our people and our very lands disappear as if they never were. We no longer fight for glory, or honor. We battle now for the right to exist."
 —General Tazri, allied commander</x:v>
       </x:c>
-      <x:c r="D6" s="20" t="str">
-        <x:v>The speaker rejects glory and honor once people and land are being erased. What remains is immediate collective action for continued existence, a narrow echo of Dune's territorial pressure and organized force.</x:v>
-      </x:c>
-      <x:c r="E6" s="20" t="str"/>
       <x:c r="F6" s="20" t="str">
         <x:v>Aurelia shows Dune at the front of the advance. General Tazri supplies the complementary reason the line holds: when both people and land can be erased, battle becomes shared territorial survival—not glory, spectacle, or aggression for its own sake.</x:v>
       </x:c>
       <x:c r="G6" s="22" t="str">
-        <x:v>SEMANTIC_REMEDIATION</x:v>
+        <x:v>RELATIONSHIP_REPLACED</x:v>
       </x:c>
       <x:c r="H6" s="20" t="str">
-        <x:v>Narrow the bridge to the already-approved direct-action and territorial-pressure facets without importing missing-color psychology.</x:v>
+        <x:v>Replace the owner-rejected Scour echo with Dune's governed card anchor and its exact land-scaled Sand-token multiplication, while preserving the boundary that the Nephilim is an anchor rather than a doctrine.</x:v>
       </x:c>
       <x:c r="I6" s="23" t="str">
-        <x:v>INSUFFICIENT_VOX_MANA_AUTHORITY_FOR_NARROW_BRIDGE</x:v>
-      </x:c>
-      <x:c r="J6" s="24" t="str"/>
+        <x:v>PASS_GOVERNED_DUNE_ANCHOR_AND_EXACT_CARD_EVIDENCE</x:v>
+      </x:c>
+      <x:c r="J6" s="24"/>
     </x:row>
     <x:row r="7" ht="94.5" customHeight="1">
       <x:c r="A7" s="21" t="str">
@@ -6947,7 +6949,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1869e1025ce743bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfacb21a8efe04546"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7142,7 +7144,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R753b0798dbd84199"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c6fc91607364855"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7340,7 +7342,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R845a6909c6724be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96ee73b27f3846c4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7533,7 +7535,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ff859882aeb47a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re760e587f86a40bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7703,7 +7705,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6155b32ff66a4dab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13c8b26ceb1f4ffc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7898,7 +7900,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72f0e4d501d14072"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cb407aa43e4c19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8091,7 +8093,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8c38ea07bbf48a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679a84b931b44005"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8286,7 +8288,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc064e254c76b4e27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cb4794478ea48e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8483,7 +8485,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b5078eec80f4122"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64749e4900694f43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8704,7 +8706,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc629c673506b4794"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc85382e986048c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8957,7 +8959,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e0a467bdbf5473a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9be277375854dfc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>